<commit_message>
replace the result order column to the db row order
</commit_message>
<xml_diff>
--- a/db.xlsx
+++ b/db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liapkin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B40BF8-5AFC-45D6-9A0C-DE4BACA13EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221E2384-6F9E-46B4-AE30-1BB50301EAEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{3AEF7474-181C-4EB9-99CA-BBDE0C603FCC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3AEF7474-181C-4EB9-99CA-BBDE0C603FCC}"/>
   </bookViews>
   <sheets>
     <sheet name="4" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -88,7 +91,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -122,7 +125,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -457,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B92C40-3444-4F44-838F-A63F47BF246F}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="8.88671875" style="1"/>
@@ -522,6 +525,966 @@
       <c r="I2" cm="1">
         <f t="array" ref="I2">SUMPRODUCT(--(MOD(C2:F2,2)&lt;&gt;0))</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C3">
+        <v>42</v>
+      </c>
+      <c r="D3">
+        <v>48</v>
+      </c>
+      <c r="E3">
+        <v>59</v>
+      </c>
+      <c r="F3">
+        <v>70</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G32" si="0">SUM(C3:F3)</f>
+        <v>219</v>
+      </c>
+      <c r="H3" cm="1">
+        <f t="array" ref="H3">SUMPRODUCT(--(MOD(C3:F3,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I3" cm="1">
+        <f t="array" ref="I3">SUMPRODUCT(--(MOD(C3:F3,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>13</v>
+      </c>
+      <c r="E4">
+        <v>27</v>
+      </c>
+      <c r="F4">
+        <v>67</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>109</v>
+      </c>
+      <c r="H4" cm="1">
+        <f t="array" ref="H4">SUMPRODUCT(--(MOD(C4:F4,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I4" cm="1">
+        <f t="array" ref="I4">SUMPRODUCT(--(MOD(C4:F4,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5">
+        <v>40</v>
+      </c>
+      <c r="E5">
+        <v>70</v>
+      </c>
+      <c r="F5">
+        <v>72</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>212</v>
+      </c>
+      <c r="H5" cm="1">
+        <f t="array" ref="H5">SUMPRODUCT(--(MOD(C5:F5,2)=0))</f>
+        <v>4</v>
+      </c>
+      <c r="I5" cm="1">
+        <f t="array" ref="I5">SUMPRODUCT(--(MOD(C5:F5,2)&lt;&gt;0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>47</v>
+      </c>
+      <c r="F6">
+        <v>50</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>103</v>
+      </c>
+      <c r="H6" cm="1">
+        <f t="array" ref="H6">SUMPRODUCT(--(MOD(C6:F6,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I6" cm="1">
+        <f t="array" ref="I6">SUMPRODUCT(--(MOD(C6:F6,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C7">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>42</v>
+      </c>
+      <c r="E7">
+        <v>47</v>
+      </c>
+      <c r="F7">
+        <v>71</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>179</v>
+      </c>
+      <c r="H7" cm="1">
+        <f t="array" ref="H7">SUMPRODUCT(--(MOD(C7:F7,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I7" cm="1">
+        <f t="array" ref="I7">SUMPRODUCT(--(MOD(C7:F7,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C8">
+        <v>37</v>
+      </c>
+      <c r="D8">
+        <v>40</v>
+      </c>
+      <c r="E8">
+        <v>48</v>
+      </c>
+      <c r="F8">
+        <v>61</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>186</v>
+      </c>
+      <c r="H8" cm="1">
+        <f t="array" ref="H8">SUMPRODUCT(--(MOD(C8:F8,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I8" cm="1">
+        <f t="array" ref="I8">SUMPRODUCT(--(MOD(C8:F8,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C9">
+        <v>25</v>
+      </c>
+      <c r="D9">
+        <v>37</v>
+      </c>
+      <c r="E9">
+        <v>45</v>
+      </c>
+      <c r="F9">
+        <v>58</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>165</v>
+      </c>
+      <c r="H9" cm="1">
+        <f t="array" ref="H9">SUMPRODUCT(--(MOD(C9:F9,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I9" cm="1">
+        <f t="array" ref="I9">SUMPRODUCT(--(MOD(C9:F9,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <v>36</v>
+      </c>
+      <c r="E10">
+        <v>45</v>
+      </c>
+      <c r="F10">
+        <v>62</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="H10" cm="1">
+        <f t="array" ref="H10">SUMPRODUCT(--(MOD(C10:F10,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I10" cm="1">
+        <f t="array" ref="I10">SUMPRODUCT(--(MOD(C10:F10,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C11">
+        <v>24</v>
+      </c>
+      <c r="D11">
+        <v>31</v>
+      </c>
+      <c r="E11">
+        <v>56</v>
+      </c>
+      <c r="F11">
+        <v>71</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>182</v>
+      </c>
+      <c r="H11" cm="1">
+        <f t="array" ref="H11">SUMPRODUCT(--(MOD(C11:F11,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I11" cm="1">
+        <f t="array" ref="I11">SUMPRODUCT(--(MOD(C11:F11,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C12">
+        <v>24</v>
+      </c>
+      <c r="D12">
+        <v>78</v>
+      </c>
+      <c r="E12">
+        <v>80</v>
+      </c>
+      <c r="F12">
+        <v>86</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>268</v>
+      </c>
+      <c r="H12" cm="1">
+        <f t="array" ref="H12">SUMPRODUCT(--(MOD(C12:F12,2)=0))</f>
+        <v>4</v>
+      </c>
+      <c r="I12" cm="1">
+        <f t="array" ref="I12">SUMPRODUCT(--(MOD(C12:F12,2)&lt;&gt;0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C13">
+        <v>19</v>
+      </c>
+      <c r="D13">
+        <v>31</v>
+      </c>
+      <c r="E13">
+        <v>34</v>
+      </c>
+      <c r="F13">
+        <v>66</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="H13" cm="1">
+        <f t="array" ref="H13">SUMPRODUCT(--(MOD(C13:F13,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I13" cm="1">
+        <f t="array" ref="I13">SUMPRODUCT(--(MOD(C13:F13,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>12</v>
+      </c>
+      <c r="F14">
+        <v>88</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>115</v>
+      </c>
+      <c r="H14" cm="1">
+        <f t="array" ref="H14">SUMPRODUCT(--(MOD(C14:F14,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I14" cm="1">
+        <f t="array" ref="I14">SUMPRODUCT(--(MOD(C14:F14,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C15">
+        <v>7</v>
+      </c>
+      <c r="D15">
+        <v>12</v>
+      </c>
+      <c r="E15">
+        <v>48</v>
+      </c>
+      <c r="F15">
+        <v>67</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>134</v>
+      </c>
+      <c r="H15" cm="1">
+        <f t="array" ref="H15">SUMPRODUCT(--(MOD(C15:F15,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I15" cm="1">
+        <f t="array" ref="I15">SUMPRODUCT(--(MOD(C15:F15,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C16">
+        <v>13</v>
+      </c>
+      <c r="D16">
+        <v>24</v>
+      </c>
+      <c r="E16">
+        <v>33</v>
+      </c>
+      <c r="F16">
+        <v>49</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>119</v>
+      </c>
+      <c r="H16" cm="1">
+        <f t="array" ref="H16">SUMPRODUCT(--(MOD(C16:F16,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I16" cm="1">
+        <f t="array" ref="I16">SUMPRODUCT(--(MOD(C16:F16,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>19</v>
+      </c>
+      <c r="F17">
+        <v>49</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>73</v>
+      </c>
+      <c r="H17" cm="1">
+        <f t="array" ref="H17">SUMPRODUCT(--(MOD(C17:F17,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I17" cm="1">
+        <f t="array" ref="I17">SUMPRODUCT(--(MOD(C17:F17,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C18">
+        <v>23</v>
+      </c>
+      <c r="D18">
+        <v>30</v>
+      </c>
+      <c r="E18">
+        <v>38</v>
+      </c>
+      <c r="F18">
+        <v>60</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>151</v>
+      </c>
+      <c r="H18" cm="1">
+        <f t="array" ref="H18">SUMPRODUCT(--(MOD(C18:F18,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I18" cm="1">
+        <f t="array" ref="I18">SUMPRODUCT(--(MOD(C18:F18,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>40</v>
+      </c>
+      <c r="E19">
+        <v>74</v>
+      </c>
+      <c r="F19">
+        <v>87</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>205</v>
+      </c>
+      <c r="H19" cm="1">
+        <f t="array" ref="H19">SUMPRODUCT(--(MOD(C19:F19,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I19" cm="1">
+        <f t="array" ref="I19">SUMPRODUCT(--(MOD(C19:F19,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C20">
+        <v>4</v>
+      </c>
+      <c r="D20">
+        <v>35</v>
+      </c>
+      <c r="E20">
+        <v>68</v>
+      </c>
+      <c r="F20">
+        <v>82</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>189</v>
+      </c>
+      <c r="H20" cm="1">
+        <f t="array" ref="H20">SUMPRODUCT(--(MOD(C20:F20,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I20" cm="1">
+        <f t="array" ref="I20">SUMPRODUCT(--(MOD(C20:F20,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C21">
+        <v>25</v>
+      </c>
+      <c r="D21">
+        <v>53</v>
+      </c>
+      <c r="E21">
+        <v>69</v>
+      </c>
+      <c r="F21">
+        <v>89</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>236</v>
+      </c>
+      <c r="H21" cm="1">
+        <f t="array" ref="H21">SUMPRODUCT(--(MOD(C21:F21,2)=0))</f>
+        <v>0</v>
+      </c>
+      <c r="I21" cm="1">
+        <f t="array" ref="I21">SUMPRODUCT(--(MOD(C21:F21,2)&lt;&gt;0))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C22">
+        <v>13</v>
+      </c>
+      <c r="D22">
+        <v>38</v>
+      </c>
+      <c r="E22">
+        <v>63</v>
+      </c>
+      <c r="F22">
+        <v>89</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>203</v>
+      </c>
+      <c r="H22" cm="1">
+        <f t="array" ref="H22">SUMPRODUCT(--(MOD(C22:F22,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I22" cm="1">
+        <f t="array" ref="I22">SUMPRODUCT(--(MOD(C22:F22,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>9</v>
+      </c>
+      <c r="E23">
+        <v>24</v>
+      </c>
+      <c r="F23">
+        <v>86</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
+      <c r="H23" cm="1">
+        <f t="array" ref="H23">SUMPRODUCT(--(MOD(C23:F23,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I23" cm="1">
+        <f t="array" ref="I23">SUMPRODUCT(--(MOD(C23:F23,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C24">
+        <v>26</v>
+      </c>
+      <c r="D24">
+        <v>34</v>
+      </c>
+      <c r="E24">
+        <v>48</v>
+      </c>
+      <c r="F24">
+        <v>72</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>180</v>
+      </c>
+      <c r="H24" cm="1">
+        <f t="array" ref="H24">SUMPRODUCT(--(MOD(C24:F24,2)=0))</f>
+        <v>4</v>
+      </c>
+      <c r="I24" cm="1">
+        <f t="array" ref="I24">SUMPRODUCT(--(MOD(C24:F24,2)&lt;&gt;0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C25">
+        <v>14</v>
+      </c>
+      <c r="D25">
+        <v>17</v>
+      </c>
+      <c r="E25">
+        <v>60</v>
+      </c>
+      <c r="F25">
+        <v>65</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>156</v>
+      </c>
+      <c r="H25" cm="1">
+        <f t="array" ref="H25">SUMPRODUCT(--(MOD(C25:F25,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I25" cm="1">
+        <f t="array" ref="I25">SUMPRODUCT(--(MOD(C25:F25,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C26">
+        <v>10</v>
+      </c>
+      <c r="D26">
+        <v>39</v>
+      </c>
+      <c r="E26">
+        <v>54</v>
+      </c>
+      <c r="F26">
+        <v>75</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>178</v>
+      </c>
+      <c r="H26" cm="1">
+        <f t="array" ref="H26">SUMPRODUCT(--(MOD(C26:F26,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I26" cm="1">
+        <f t="array" ref="I26">SUMPRODUCT(--(MOD(C26:F26,2)&lt;&gt;0))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C27">
+        <v>31</v>
+      </c>
+      <c r="D27">
+        <v>35</v>
+      </c>
+      <c r="E27">
+        <v>45</v>
+      </c>
+      <c r="F27">
+        <v>53</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>164</v>
+      </c>
+      <c r="H27" cm="1">
+        <f t="array" ref="H27">SUMPRODUCT(--(MOD(C27:F27,2)=0))</f>
+        <v>0</v>
+      </c>
+      <c r="I27" cm="1">
+        <f t="array" ref="I27">SUMPRODUCT(--(MOD(C27:F27,2)&lt;&gt;0))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C28">
+        <v>19</v>
+      </c>
+      <c r="D28">
+        <v>43</v>
+      </c>
+      <c r="E28">
+        <v>55</v>
+      </c>
+      <c r="F28">
+        <v>56</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>173</v>
+      </c>
+      <c r="H28" cm="1">
+        <f t="array" ref="H28">SUMPRODUCT(--(MOD(C28:F28,2)=0))</f>
+        <v>1</v>
+      </c>
+      <c r="I28" cm="1">
+        <f t="array" ref="I28">SUMPRODUCT(--(MOD(C28:F28,2)&lt;&gt;0))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C29">
+        <v>3</v>
+      </c>
+      <c r="D29">
+        <v>10</v>
+      </c>
+      <c r="E29">
+        <v>52</v>
+      </c>
+      <c r="F29">
+        <v>88</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>153</v>
+      </c>
+      <c r="H29" cm="1">
+        <f t="array" ref="H29">SUMPRODUCT(--(MOD(C29:F29,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I29" cm="1">
+        <f t="array" ref="I29">SUMPRODUCT(--(MOD(C29:F29,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C30">
+        <v>22</v>
+      </c>
+      <c r="D30">
+        <v>50</v>
+      </c>
+      <c r="E30">
+        <v>66</v>
+      </c>
+      <c r="F30">
+        <v>85</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>223</v>
+      </c>
+      <c r="H30" cm="1">
+        <f t="array" ref="H30">SUMPRODUCT(--(MOD(C30:F30,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I30" cm="1">
+        <f t="array" ref="I30">SUMPRODUCT(--(MOD(C30:F30,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C31">
+        <v>34</v>
+      </c>
+      <c r="D31">
+        <v>56</v>
+      </c>
+      <c r="E31">
+        <v>71</v>
+      </c>
+      <c r="F31">
+        <v>82</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>243</v>
+      </c>
+      <c r="H31" cm="1">
+        <f t="array" ref="H31">SUMPRODUCT(--(MOD(C31:F31,2)=0))</f>
+        <v>3</v>
+      </c>
+      <c r="I31" cm="1">
+        <f t="array" ref="I31">SUMPRODUCT(--(MOD(C31:F31,2)&lt;&gt;0))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1">
+        <v>46132</v>
+      </c>
+      <c r="C32">
+        <v>15</v>
+      </c>
+      <c r="D32">
+        <v>66</v>
+      </c>
+      <c r="E32">
+        <v>83</v>
+      </c>
+      <c r="F32">
+        <v>88</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="0"/>
+        <v>252</v>
+      </c>
+      <c r="H32" cm="1">
+        <f t="array" ref="H32">SUMPRODUCT(--(MOD(C32:F32,2)=0))</f>
+        <v>2</v>
+      </c>
+      <c r="I32" cm="1">
+        <f t="array" ref="I32">SUMPRODUCT(--(MOD(C32:F32,2)&lt;&gt;0))</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>